<commit_message>
feat: ra mat Web App Quan Ly Cong Viec dong bo 2 chieu Google Sheets va UI/UX Linear SaaS
</commit_message>
<xml_diff>
--- a/Quan_Ly_Cong_Viec_KingBlue.xlsx
+++ b/Quan_Ly_Cong_Viec_KingBlue.xlsx
@@ -125,7 +125,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -147,11 +147,44 @@
         <color rgb="00CBD5E0"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -202,6 +235,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -595,7 +629,7 @@
           <t>TỔNG SỐ CÔNG VIỆC</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n"/>
+      <c r="C4" s="20" t="n"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>HOÀN THÀNH</t>
@@ -621,14 +655,14 @@
           <t>TỶ LỆ HOÀN THÀNH</t>
         </is>
       </c>
-      <c r="I4" s="3" t="n"/>
+      <c r="I4" s="20" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="4">
         <f>COUNTA('DS CONG VIEC'!B5:B100)</f>
         <v/>
       </c>
-      <c r="C5" s="3" t="n"/>
+      <c r="C5" s="20" t="n"/>
       <c r="D5" s="4">
         <f>COUNTIF('DS CONG VIEC'!I5:I100, "Hoàn thành")</f>
         <v/>
@@ -649,7 +683,7 @@
         <f>IF(B5&gt;0, D5/B5, 0)</f>
         <v/>
       </c>
-      <c r="I5" s="3" t="n"/>
+      <c r="I5" s="20" t="n"/>
     </row>
     <row r="7">
       <c r="B7" s="6" t="inlineStr">
@@ -1095,11 +1129,11 @@
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="D4"/>
+    <mergeCell ref="F4"/>
+    <mergeCell ref="E4"/>
+    <mergeCell ref="G4"/>
+    <mergeCell ref="B5:C5"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="E4"/>
-    <mergeCell ref="F4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="G4"/>
     <mergeCell ref="A1:I2"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H4:I4"/>
@@ -1122,7 +1156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1229,809 +1263,205 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-01</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Quay video test tải máy khoan pin KM18QE</t>
-        </is>
-      </c>
-      <c r="D5" s="8" t="inlineStr">
-        <is>
-          <t>YouTube / Video</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Tứ</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>Kiều Thương</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-02</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="K5" s="9">
-        <f>IF(I5="Hoàn thành", "Đã xong", IF(ISBLANK(H5), "", IF(H5&lt;TODAY(), "Quá hạn", IF(H5-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L5" s="15" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/...</t>
-        </is>
-      </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>Chuẩn bị mẫu bê tông và đá mài</t>
-        </is>
-      </c>
+      <c r="A5" s="11" t="n"/>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="8" t="n"/>
+      <c r="D5" s="8" t="n"/>
+      <c r="E5" s="8" t="n"/>
+      <c r="F5" s="8" t="n"/>
+      <c r="G5" s="11" t="n"/>
+      <c r="H5" s="11" t="n"/>
+      <c r="I5" s="13" t="n"/>
+      <c r="J5" s="14" t="n"/>
+      <c r="K5" s="9" t="n"/>
+      <c r="L5" s="15" t="n"/>
+      <c r="M5" s="8" t="n"/>
+      <c r="N5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-02</t>
-        </is>
-      </c>
-      <c r="C6" s="8" t="inlineStr">
-        <is>
-          <t>Chụp ảnh sản phẩm thùng đồ nghề KHD4233</t>
-        </is>
-      </c>
-      <c r="D6" s="8" t="inlineStr">
-        <is>
-          <t>Thiết kế &amp; Media</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Tứ</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Thiện</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="I6" s="16" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="J6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="9">
-        <f>IF(I6="Hoàn thành", "Đã xong", IF(ISBLANK(H6), "", IF(H6&lt;TODAY(), "Quá hạn", IF(H6-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L6" s="15" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="M6" s="8" t="inlineStr">
-        <is>
-          <t>https://drive.google.com/...</t>
-        </is>
-      </c>
-      <c r="N6" s="8" t="inlineStr">
-        <is>
-          <t>Đã retouched xong 8 góc ảnh</t>
-        </is>
-      </c>
+      <c r="A6" s="11" t="n"/>
+      <c r="B6" s="11" t="n"/>
+      <c r="C6" s="8" t="n"/>
+      <c r="D6" s="8" t="n"/>
+      <c r="E6" s="8" t="n"/>
+      <c r="F6" s="8" t="n"/>
+      <c r="G6" s="11" t="n"/>
+      <c r="H6" s="11" t="n"/>
+      <c r="I6" s="16" t="n"/>
+      <c r="J6" s="14" t="n"/>
+      <c r="K6" s="9" t="n"/>
+      <c r="L6" s="15" t="n"/>
+      <c r="M6" s="8" t="n"/>
+      <c r="N6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-03</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Thiết kế banner &amp; poster sự kiện triển lãm Vietbuild</t>
-        </is>
-      </c>
-      <c r="D7" s="8" t="inlineStr">
-        <is>
-          <t>Trade &amp; POSM Đại lý</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
-        <is>
-          <t>Thiện</t>
-        </is>
-      </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>Thụy Thương</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-09</t>
-        </is>
-      </c>
-      <c r="I7" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J7" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="K7" s="9">
-        <f>IF(I7="Hoàn thành", "Đã xong", IF(ISBLANK(H7), "", IF(H7&lt;TODAY(), "Quá hạn", IF(H7-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L7" s="17" t="inlineStr">
-        <is>
-          <t>Khẩn cấp</t>
-        </is>
-      </c>
-      <c r="M7" s="8" t="inlineStr">
-        <is>
-          <t>file:///Users/Admin/Documents/...</t>
-        </is>
-      </c>
-      <c r="N7" s="8" t="inlineStr">
-        <is>
-          <t>Đang duyệt layout 3 phương án</t>
-        </is>
-      </c>
+      <c r="A7" s="11" t="n"/>
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="11" t="n"/>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="14" t="n"/>
+      <c r="K7" s="9" t="n"/>
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="8" t="n"/>
+      <c r="N7" s="8" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-04</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Viết bài chuẩn SEO giới thiệu công nghệ Brushless Motor</t>
-        </is>
-      </c>
-      <c r="D8" s="8" t="inlineStr">
-        <is>
-          <t>Website &amp; SEO</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>Hoài Thương</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>Admin</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="J8" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="9">
-        <f>IF(I8="Hoàn thành", "Đã xong", IF(ISBLANK(H8), "", IF(H8&lt;TODAY(), "Quá hạn", IF(H8-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L8" s="15" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="M8" s="8" t="inlineStr">
-        <is>
-          <t>https://kingblue.vn/tin-tuc</t>
-        </is>
-      </c>
-      <c r="N8" s="8" t="inlineStr">
-        <is>
-          <t>Đã index Google</t>
-        </is>
-      </c>
+      <c r="A8" s="11" t="n"/>
+      <c r="B8" s="11" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="11" t="n"/>
+      <c r="I8" s="16" t="n"/>
+      <c r="J8" s="14" t="n"/>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="15" t="n"/>
+      <c r="M8" s="8" t="n"/>
+      <c r="N8" s="8" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-05</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Lên kịch bản &amp; liên hệ KOC test cờ lê lực King Blue</t>
-        </is>
-      </c>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>TikTok &amp; KOC</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
-        <is>
-          <t>Kiều Thương</t>
-        </is>
-      </c>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Tứ</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-10</t>
-        </is>
-      </c>
-      <c r="I9" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="K9" s="9">
-        <f>IF(I9="Hoàn thành", "Đã xong", IF(ISBLANK(H9), "", IF(H9&lt;TODAY(), "Quá hạn", IF(H9-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L9" s="15" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="M9" s="8" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/...</t>
-        </is>
-      </c>
-      <c r="N9" s="8" t="inlineStr">
-        <is>
-          <t>Đã gửi tin nhắn cho 3 KOC ngành cơ khí</t>
-        </is>
-      </c>
+      <c r="A9" s="11" t="n"/>
+      <c r="B9" s="11" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="11" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" s="14" t="n"/>
+      <c r="K9" s="9" t="n"/>
+      <c r="L9" s="15" t="n"/>
+      <c r="M9" s="8" t="n"/>
+      <c r="N9" s="8" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-06</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>Cập nhật giá niêm yết và khuyến mãi đại lý lên kingtools.vn</t>
-        </is>
-      </c>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Sàn TMĐT (Shopee/Lazada)</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
-        <is>
-          <t>Thức</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Ngân</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="I10" s="18" t="inlineStr">
-        <is>
-          <t>Đang duyệt</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="K10" s="9">
-        <f>IF(I10="Hoàn thành", "Đã xong", IF(ISBLANK(H10), "", IF(H10&lt;TODAY(), "Quá hạn", IF(H10-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L10" s="15" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="M10" s="8" t="inlineStr">
-        <is>
-          <t>https://kingtools.vn/...</t>
-        </is>
-      </c>
-      <c r="N10" s="8" t="inlineStr">
-        <is>
-          <t>Chờ Giám đốc ký duyệt chính sách</t>
-        </is>
-      </c>
+      <c r="A10" s="11" t="n"/>
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="18" t="n"/>
+      <c r="J10" s="14" t="n"/>
+      <c r="K10" s="9" t="n"/>
+      <c r="L10" s="15" t="n"/>
+      <c r="M10" s="8" t="n"/>
+      <c r="N10" s="8" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-07</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Thiết kế quầy kệ trưng bày POSM nhận diện cho Đại lý Cấp 1</t>
-        </is>
-      </c>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Trade &amp; POSM Đại lý</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
-        <is>
-          <t>Thiện</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="inlineStr">
-        <is>
-          <t>Thức</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-28</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="I11" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K11" s="9">
-        <f>IF(I11="Hoàn thành", "Đã xong", IF(ISBLANK(H11), "", IF(H11&lt;TODAY(), "Quá hạn", IF(H11-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L11" s="17" t="inlineStr">
-        <is>
-          <t>Khẩn cấp</t>
-        </is>
-      </c>
-      <c r="M11" s="8" t="inlineStr">
-        <is>
-          <t>file:///Users/Admin/Documents/...</t>
-        </is>
-      </c>
-      <c r="N11" s="8" t="inlineStr">
-        <is>
-          <t>Xưởng đang gửi báo giá đóng kệ</t>
-        </is>
-      </c>
+      <c r="A11" s="11" t="n"/>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="13" t="n"/>
+      <c r="J11" s="14" t="n"/>
+      <c r="K11" s="9" t="n"/>
+      <c r="L11" s="17" t="n"/>
+      <c r="M11" s="8" t="n"/>
+      <c r="N11" s="8" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-08</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Đăng bài Fanpage: Mẹo sử dụng đá cắt an toàn &amp; tặng mã voucher</t>
-        </is>
-      </c>
-      <c r="D12" s="8" t="inlineStr">
-        <is>
-          <t>Facebook Fanpage</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>Hoài Thương</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>Thiện</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="I12" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K12" s="9">
-        <f>IF(I12="Hoàn thành", "Đã xong", IF(ISBLANK(H12), "", IF(H12&lt;TODAY(), "Quá hạn", IF(H12-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L12" s="15" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="M12" s="8" t="inlineStr">
-        <is>
-          <t>https://facebook.com/KingBlue-tools...</t>
-        </is>
-      </c>
-      <c r="N12" s="8" t="inlineStr">
-        <is>
-          <t>Đã xong visual, chờ giờ vàng lên bài</t>
-        </is>
-      </c>
+      <c r="A12" s="11" t="n"/>
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="n"/>
+      <c r="I12" s="13" t="n"/>
+      <c r="J12" s="14" t="n"/>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="15" t="n"/>
+      <c r="M12" s="8" t="n"/>
+      <c r="N12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-09</t>
-        </is>
-      </c>
-      <c r="C13" s="8" t="inlineStr">
-        <is>
-          <t>Trực chat sàn &amp; tối ưu giỏ hàng TikTok Shop</t>
-        </is>
-      </c>
-      <c r="D13" s="8" t="inlineStr">
-        <is>
-          <t>Sàn TMĐT (Shopee/Lazada)</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
-        <is>
-          <t>Ngân</t>
-        </is>
-      </c>
-      <c r="F13" s="8" t="inlineStr">
-        <is>
-          <t>Thức</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>2026-09-29</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="I13" s="16" t="inlineStr">
-        <is>
-          <t>Hoàn thành</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="9">
-        <f>IF(I13="Hoàn thành", "Đã xong", IF(ISBLANK(H13), "", IF(H13&lt;TODAY(), "Quá hạn", IF(H13-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L13" s="15" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="M13" s="8" t="inlineStr">
-        <is>
-          <t>https://shopee.vn/...</t>
-        </is>
-      </c>
-      <c r="N13" s="8" t="inlineStr">
-        <is>
-          <t>Tỷ lệ phản hồi chat đạt 98%</t>
-        </is>
-      </c>
+      <c r="A13" s="11" t="n"/>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="16" t="n"/>
+      <c r="J13" s="14" t="n"/>
+      <c r="K13" s="9" t="n"/>
+      <c r="L13" s="15" t="n"/>
+      <c r="M13" s="8" t="n"/>
+      <c r="N13" s="8" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-10</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Soạn nội dung cẩm nang sản phẩm &amp; chính sách đại lý</t>
-        </is>
-      </c>
-      <c r="D14" s="8" t="inlineStr">
-        <is>
-          <t>Trade &amp; POSM Đại lý</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
-        <is>
-          <t>Thụy Thương</t>
-        </is>
-      </c>
-      <c r="F14" s="8" t="inlineStr">
-        <is>
-          <t>Hoài Thương</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-03</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="I14" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J14" s="14" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="K14" s="9">
-        <f>IF(I14="Hoàn thành", "Đã xong", IF(ISBLANK(H14), "", IF(H14&lt;TODAY(), "Quá hạn", IF(H14-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L14" s="15" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="M14" s="8" t="inlineStr">
-        <is>
-          <t>https://docs.google.com/...</t>
-        </is>
-      </c>
-      <c r="N14" s="8" t="inlineStr">
-        <is>
-          <t>Đang rà soát danh mục máy pin</t>
-        </is>
-      </c>
+      <c r="A14" s="11" t="n"/>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="11" t="n"/>
+      <c r="H14" s="11" t="n"/>
+      <c r="I14" s="13" t="n"/>
+      <c r="J14" s="14" t="n"/>
+      <c r="K14" s="9" t="n"/>
+      <c r="L14" s="15" t="n"/>
+      <c r="M14" s="8" t="n"/>
+      <c r="N14" s="8" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-11</t>
-        </is>
-      </c>
-      <c r="C15" s="8" t="inlineStr">
-        <is>
-          <t>Đóng gói 50 đơn hàng combo máy pin ra mắt (Kho Nam)</t>
-        </is>
-      </c>
-      <c r="D15" s="8" t="inlineStr">
-        <is>
-          <t>Sàn TMĐT (Shopee/Lazada)</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>Hùng</t>
-        </is>
-      </c>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Thức</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-05</t>
-        </is>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="I15" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J15" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="K15" s="9">
-        <f>IF(I15="Hoàn thành", "Đã xong", IF(ISBLANK(H15), "", IF(H15&lt;TODAY(), "Quá hạn", IF(H15-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L15" s="15" t="inlineStr">
-        <is>
-          <t>Cao</t>
-        </is>
-      </c>
-      <c r="M15" s="8" t="inlineStr">
-        <is>
-          <t>file:///Users/Admin/Documents/...</t>
-        </is>
-      </c>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>Đã dán tem bảo hành và đóng thùng</t>
-        </is>
-      </c>
+      <c r="A15" s="11" t="n"/>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="11" t="n"/>
+      <c r="I15" s="13" t="n"/>
+      <c r="J15" s="14" t="n"/>
+      <c r="K15" s="9" t="n"/>
+      <c r="L15" s="15" t="n"/>
+      <c r="M15" s="8" t="n"/>
+      <c r="N15" s="8" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>KB-MKT-12</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Kiểm kê vật tư bao bì &amp; đóng gói hàng kho Miền Bắc</t>
-        </is>
-      </c>
-      <c r="D16" s="8" t="inlineStr">
-        <is>
-          <t>Sàn TMĐT (Shopee/Lazada)</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
-        <is>
-          <t>Hùng Miền Bắc</t>
-        </is>
-      </c>
-      <c r="F16" s="8" t="inlineStr">
-        <is>
-          <t>Ngân</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-04</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>2026-10-07</t>
-        </is>
-      </c>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>Đang làm</t>
-        </is>
-      </c>
-      <c r="J16" s="14" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K16" s="9">
-        <f>IF(I16="Hoàn thành", "Đã xong", IF(ISBLANK(H16), "", IF(H16&lt;TODAY(), "Quá hạn", IF(H16-TODAY()&lt;=2, "Sắp đến hạn", "Đúng hạn"))))</f>
-        <v/>
-      </c>
-      <c r="L16" s="15" t="inlineStr">
-        <is>
-          <t>Trung bình</t>
-        </is>
-      </c>
-      <c r="M16" s="8" t="inlineStr">
-        <is>
-          <t>file:///Users/Admin/Documents/...</t>
-        </is>
-      </c>
-      <c r="N16" s="8" t="inlineStr">
-        <is>
-          <t>Bổ sung thùng carton cỡ M &amp; màng co</t>
-        </is>
-      </c>
-    </row>
+      <c r="A16" s="11" t="n"/>
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="11" t="n"/>
+      <c r="I16" s="13" t="n"/>
+      <c r="J16" s="14" t="n"/>
+      <c r="K16" s="9" t="n"/>
+      <c r="L16" s="15" t="n"/>
+      <c r="M16" s="8" t="n"/>
+      <c r="N16" s="8" t="n"/>
+    </row>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:N2"/>

</xml_diff>